<commit_message>
Changed bib labels, new references, advance in literature review and managed to put table into pdf
</commit_message>
<xml_diff>
--- a/thesis/data/table_literature_review.xlsx
+++ b/thesis/data/table_literature_review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mateo\Documents\Universidad\Master\Thesis\BEReBASL\thesis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C71D36AC-C6C5-49E8-BDF6-2268837DBE54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B1D8F4-4D95-4C80-9875-71E7B245E65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D47D74D5-B8DF-4140-AD42-DCD0A14E194D}"/>
   </bookViews>
@@ -40,23 +40,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="41">
   <si>
     <t>Reference</t>
   </si>
   <si>
-    <t>Dynamic perspective</t>
-  </si>
-  <si>
     <t>Distributional assumptions, sample of reject region or experts judgement</t>
   </si>
   <si>
-    <t>Concludes RI can (reliably) work?</t>
-  </si>
-  <si>
-    <t>Only with full sample of reject region</t>
-  </si>
-  <si>
     <t>Estimation of $p(x)$ for further usage in EM based methods</t>
   </si>
   <si>
@@ -72,9 +63,6 @@
     <t>HandHanley1993CanRIWork</t>
   </si>
   <si>
-    <t>Reliability of causality and dimensionality</t>
-  </si>
-  <si>
     <t>Knowledge and existence of causal non-cyclic relationships between features</t>
   </si>
   <si>
@@ -90,12 +78,6 @@
     <t>Rejects guide the decision boundary through low density regions in the features space</t>
   </si>
   <si>
-    <t>High dimensional feature space problematic</t>
-  </si>
-  <si>
-    <t>Yes, evaluation method is unreliable</t>
-  </si>
-  <si>
     <t>Low density regions of features space aligned with known labels separation</t>
   </si>
   <si>
@@ -105,27 +87,15 @@
     <t>Label missingness be independent across observations</t>
   </si>
   <si>
-    <t>Independence condition is illogical in dynamic context, numerical problems</t>
-  </si>
-  <si>
     <t>Estimation of unconditional means of features and probability of reject</t>
   </si>
   <si>
-    <t>Yes, in theoretical and simulation based results</t>
-  </si>
-  <si>
     <t>Banasik01032010</t>
   </si>
   <si>
-    <t>No, maybe with high rejection rates</t>
-  </si>
-  <si>
     <t>Augmentation via reweighting using accepts rejects model</t>
   </si>
   <si>
-    <t>Augmentation is not adequate for RI</t>
-  </si>
-  <si>
     <t>RI approach</t>
   </si>
   <si>
@@ -138,31 +108,61 @@
     <t>Accept reject model estimable</t>
   </si>
   <si>
-    <t>Assumptions explicit?</t>
-  </si>
-  <si>
-    <t>Theoretical/heuristic justification?</t>
-  </si>
-  <si>
-    <t>Infers Rejects label for evaluation?</t>
-  </si>
-  <si>
-    <t>Type of result</t>
-  </si>
-  <si>
-    <t>Theoretical</t>
-  </si>
-  <si>
-    <t>Empirical</t>
-  </si>
-  <si>
-    <t>Theoretical and simulation</t>
+    <t>Anderson2019BayesianNetForRI</t>
+  </si>
+  <si>
+    <t>LiEtAl2017SemisupervisedSVM</t>
+  </si>
+  <si>
+    <t>BuckerEtAl2013MNARRI</t>
   </si>
   <si>
     <t>Yes</t>
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>Result type</t>
+  </si>
+  <si>
+    <t>Does RI work?</t>
+  </si>
+  <si>
+    <t>Only with labeled rejects' smaple</t>
+  </si>
+  <si>
+    <t>Augmentation inadequate for RI</t>
+  </si>
+  <si>
+    <t>High dimensional feature space</t>
+  </si>
+  <si>
+    <t>Reliability of causality, dimensionality</t>
+  </si>
+  <si>
+    <t>Dynamic persp.</t>
+  </si>
+  <si>
+    <t>Theor.</t>
+  </si>
+  <si>
+    <t>Emp.</t>
+  </si>
+  <si>
+    <t>Theor., sim.</t>
+  </si>
+  <si>
+    <t>Theo./ heur. justified?</t>
+  </si>
+  <si>
+    <t>Assump. explicit?</t>
+  </si>
+  <si>
+    <t>Infers Rejects' label for eval?</t>
+  </si>
+  <si>
+    <t>Independence condition\footnote{The condition comes from the cited paper \cite{BuckerKramer2011} in the proof} illogical in dynamic context, numerical problems</t>
   </si>
 </sst>
 </file>
@@ -206,10 +206,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -565,74 +568,74 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="C1" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" t="s">
+        <v>39</v>
+      </c>
+      <c r="G1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" t="s">
+        <v>3</v>
+      </c>
+      <c r="J1" t="s">
         <v>33</v>
-      </c>
-      <c r="F1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G1" t="s">
-        <v>35</v>
-      </c>
-      <c r="H1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>
       </c>
-      <c r="E2" t="b">
+      <c r="E2" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>40</v>
+      <c r="F2" t="b">
+        <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J2" t="b">
+      <c r="J2" s="1" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="C3" s="2" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
@@ -640,17 +643,17 @@
       <c r="E3" t="b">
         <v>0</v>
       </c>
-      <c r="F3" t="s">
-        <v>40</v>
+      <c r="F3" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>37</v>
-      </c>
-      <c r="H3" t="s">
-        <v>13</v>
+        <v>35</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="J3" s="1" t="b">
         <v>0</v>
@@ -658,45 +661,45 @@
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>35</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F4" t="s">
-        <v>39</v>
-      </c>
-      <c r="G4" t="s">
-        <v>37</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J4" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>20</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
@@ -704,31 +707,31 @@
       <c r="E5" t="b">
         <v>1</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="G5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I5" s="2" t="s">
+      <c r="J5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="J5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>31</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
@@ -736,17 +739,17 @@
       <c r="E6" t="b">
         <v>1</v>
       </c>
-      <c r="F6" t="s">
-        <v>40</v>
+      <c r="F6" t="b">
+        <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J6" t="b">
         <v>0</v>
@@ -755,11 +758,18 @@
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
     </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="D10" s="1"/>
+    </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="E11" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -776,32 +786,32 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Further work on the literature, changes in reference labels for consistency
</commit_message>
<xml_diff>
--- a/thesis/data/table_literature_review.xlsx
+++ b/thesis/data/table_literature_review.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mateo\Documents\Universidad\Master\Thesis\BEReBASL\thesis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82B1D8F4-4D95-4C80-9875-71E7B245E65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B2CA311-2D5D-4CF8-A87F-C14458726491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D47D74D5-B8DF-4140-AD42-DCD0A14E194D}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="68">
   <si>
     <t>Reference</t>
   </si>
@@ -57,57 +56,24 @@
     <t>Economic costs of sample</t>
   </si>
   <si>
-    <t>Anderson2019_BayesianNetForRI</t>
-  </si>
-  <si>
     <t>HandHanley1993CanRIWork</t>
   </si>
   <si>
     <t>Knowledge and existence of causal non-cyclic relationships between features</t>
   </si>
   <si>
-    <t>Extrapolation to rejects through bayesian network, then build scorecard on augemented sample</t>
-  </si>
-  <si>
     <t>Moderately</t>
   </si>
   <si>
-    <t>Li_et_al_2017_semisupervised_svm</t>
-  </si>
-  <si>
-    <t>Rejects guide the decision boundary through low density regions in the features space</t>
-  </si>
-  <si>
-    <t>Low density regions of features space aligned with known labels separation</t>
-  </si>
-  <si>
-    <t>Bucker_etal_2013_MNAR_RI</t>
-  </si>
-  <si>
-    <t>Label missingness be independent across observations</t>
-  </si>
-  <si>
-    <t>Estimation of unconditional means of features and probability of reject</t>
-  </si>
-  <si>
     <t>Banasik01032010</t>
   </si>
   <si>
-    <t>Augmentation via reweighting using accepts rejects model</t>
-  </si>
-  <si>
-    <t>RI approach</t>
-  </si>
-  <si>
     <t>RI Approach</t>
   </si>
   <si>
     <t>Key identifying assumptions</t>
   </si>
   <si>
-    <t>Accept reject model estimable</t>
-  </si>
-  <si>
     <t>Anderson2019BayesianNetForRI</t>
   </si>
   <si>
@@ -144,15 +110,9 @@
     <t>Dynamic persp.</t>
   </si>
   <si>
-    <t>Theor.</t>
-  </si>
-  <si>
     <t>Emp.</t>
   </si>
   <si>
-    <t>Theor., sim.</t>
-  </si>
-  <si>
     <t>Theo./ heur. justified?</t>
   </si>
   <si>
@@ -163,6 +123,126 @@
   </si>
   <si>
     <t>Independence condition\footnote{The condition comes from the cited paper \cite{BuckerKramer2011} in the proof} illogical in dynamic context, numerical problems</t>
+  </si>
+  <si>
+    <t>Theo.</t>
+  </si>
+  <si>
+    <t>Theo., sim.</t>
+  </si>
+  <si>
+    <t>BanasikCrook2003SampleSelBias</t>
+  </si>
+  <si>
+    <t>Emp., sim.</t>
+  </si>
+  <si>
+    <t>Moderately if MNAR and conservative FI</t>
+  </si>
+  <si>
+    <t>Errors in modelled equations are correlated, knowledge of relevant variables</t>
+  </si>
+  <si>
+    <t>Bivariate Probit for PD and AR equations (BVP)</t>
+  </si>
+  <si>
+    <t>BVP, Augmentation and BVP with Augmentation</t>
+  </si>
+  <si>
+    <t>Accept reject model estimable, enough rare accepts to correct</t>
+  </si>
+  <si>
+    <t>Augmentation via reweighting using AR model</t>
+  </si>
+  <si>
+    <t>Identification of AR and PD equations, correlation between their errors being $&gt;0$</t>
+  </si>
+  <si>
+    <t>No, worse than only accepts</t>
+  </si>
+  <si>
+    <t>bansikCrook2007</t>
+  </si>
+  <si>
+    <t>CrookBanasik2004DoesRIimprove</t>
+  </si>
+  <si>
+    <t>Augmentation and Extrapolation</t>
+  </si>
+  <si>
+    <t>Extrapolation to rejects through bayesian network, then build scorecard on extrapolated sample</t>
+  </si>
+  <si>
+    <t>MancisdorEtAl2020DeepGenMForRI</t>
+  </si>
+  <si>
+    <t>Use a generative model with latent features $L$\footnote{They use $z$ as letter in the paper, but here that letter stands for the acceptance status and is thus changed} in form $Y \to L \to X$, where rejects are used to train the encoder of $X$ onto $L$, while being tied by the accepts to be consistent in class conditional prior assumptions $Y \to L$</t>
+  </si>
+  <si>
+    <t>Causal markov chain $Y \to Z \to X$, distributional assumptions on certain marginals of the system. Implicitly MAR\footnote{Effecitvely they model $P(Y | X, Z=a) = P(Y | X, Z = r)$ assumption}</t>
+  </si>
+  <si>
+    <t>Numerical stability, sensitivity to initial weights, explainability for regulatory</t>
+  </si>
+  <si>
+    <t>ShengEtAl2024RICostSenstiveJointDistAdap</t>
+  </si>
+  <si>
+    <t>Semisupervised SVM (S3VM): Rejects guide the decision boundary through low density regions in the features space</t>
+  </si>
+  <si>
+    <t>Estimation of unconditional means of features and probability of reject for generative model</t>
+  </si>
+  <si>
+    <t>For Joint Distribution Adaptation (JDA) to reduce dist. Differences between rejects and accepts, and for cost sensitive S3VM</t>
+  </si>
+  <si>
+    <t>Low density regions of features space aligned with known labels separation, MAR</t>
+  </si>
+  <si>
+    <t>Label missingness be independent across observations, MNAR</t>
+  </si>
+  <si>
+    <t>JDA can turn MNAR into MAR in latent space, low density separability assumption</t>
+  </si>
+  <si>
+    <t>JDA depends on high feature dimensionality, computational costs, explaniability</t>
+  </si>
+  <si>
+    <t>Feelders2000RIMixtureModels</t>
+  </si>
+  <si>
+    <t>MAR</t>
+  </si>
+  <si>
+    <t>EM algorithm, for rejects explicit expectation over the two classes weighted by the posterior</t>
+  </si>
+  <si>
+    <t>Sim.</t>
+  </si>
+  <si>
+    <t>Parameters scale quadratically with features dimensionality, doubtful whether the DGP can be so simple and unrealistic acceptance rule</t>
+  </si>
+  <si>
+    <t>Yes, for small samples and feature space</t>
+  </si>
+  <si>
+    <t>BoyesHoffmann1985HeckmanInCreditScoring</t>
+  </si>
+  <si>
+    <t>MNAR, Bivariate Probit assumptions, FI are rational and may seek to optimize for high balances</t>
+  </si>
+  <si>
+    <t>Emp. and simulation</t>
+  </si>
+  <si>
+    <t>Unclear, only comparision of decision differences presented</t>
+  </si>
+  <si>
+    <t>Data required for proposed ``behavioral" credit scoring model is hard to obtain</t>
+  </si>
+  <si>
+    <t>Heckman type PD/AR estimation with augmentation where weights are proportional to population frequencies for behavioral scoring model</t>
   </si>
 </sst>
 </file>
@@ -549,10 +629,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8852FF5C-5175-44DA-A620-18833DBB2C7A}">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.33203125" customWidth="1"/>
     <col min="2" max="3" width="28.21875" customWidth="1"/>
     <col min="4" max="4" width="21.88671875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.6640625" customWidth="1"/>
@@ -568,36 +648,36 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C1" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D1" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="F1" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="G1" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="H1" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="I1" t="s">
         <v>3</v>
       </c>
       <c r="J1" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>2</v>
@@ -615,10 +695,10 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>4</v>
@@ -629,63 +709,63 @@
     </row>
     <row r="3" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D3" t="b">
-        <v>1</v>
-      </c>
-      <c r="E3" t="b">
-        <v>0</v>
-      </c>
-      <c r="F3" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="G3" t="s">
-        <v>35</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>9</v>
-      </c>
       <c r="I3" s="2" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="J3" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" t="s">
-        <v>35</v>
-      </c>
       <c r="H4" s="2" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="J4" t="b">
         <v>0</v>
@@ -693,31 +773,31 @@
     </row>
     <row r="5" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" t="s">
         <v>14</v>
       </c>
-      <c r="D5" t="b">
-        <v>1</v>
-      </c>
-      <c r="E5" t="b">
-        <v>1</v>
-      </c>
-      <c r="F5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" t="s">
-        <v>25</v>
-      </c>
       <c r="I5" s="2" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="J5" t="b">
         <v>0</v>
@@ -725,13 +805,13 @@
     </row>
     <row r="6" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
@@ -743,78 +823,254 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="J6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="1"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="C9" s="1"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="E11" s="1"/>
+      <c r="C8" s="2" t="str">
+        <f>"For BVP like in \textcite{"&amp;A7&amp;"}. For Augmentation like \textcite{"&amp;A6&amp;"}"</f>
+        <v>For BVP like in \textcite{BanasikCrook2003SampleSelBias}. For Augmentation like \textcite{Banasik01032010}</v>
+      </c>
+      <c r="D8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" t="s">
+        <v>23</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" s="2" t="str">
+        <f>"Also alike to \textcite{"&amp;A7&amp;"} and \textcite{"&amp;A6&amp;"}"</f>
+        <v>Also alike to \textcite{BanasikCrook2003SampleSelBias} and \textcite{Banasik01032010}</v>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="2" t="str">
+        <f>"For Augmentation like \textcite{"&amp;A6&amp;"}, for extrapolation $\mathbb{P}(Y=g | X)$ similar in accepts and rejects"</f>
+        <v>For Augmentation like \textcite{Banasik01032010}, for extrapolation $\mathbb{P}(Y=g | X)$ similar in accepts and rejects</v>
+      </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9" t="s">
+        <v>23</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" s="1" t="str">
+        <f>"Like \textcite{"&amp;A7&amp;"} and \textcite{"&amp;A6&amp;"}"</f>
+        <v>Like \textcite{BanasikCrook2003SampleSelBias} and \textcite{Banasik01032010}</v>
+      </c>
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" t="s">
+        <v>23</v>
+      </c>
+      <c r="H10" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="J10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" t="s">
+        <v>23</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" t="s">
+        <v>59</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="J12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" t="b">
+        <v>0</v>
+      </c>
+      <c r="G13" t="s">
+        <v>64</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="J13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="J14" s="1"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C15" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD0A6221-C3E5-43E7-83EA-25D1D90EAB9E}">
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Almost final - only need to check last row
</commit_message>
<xml_diff>
--- a/thesis/data/table_literature_review.xlsx
+++ b/thesis/data/table_literature_review.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mateo\Documents\Universidad\Master\Thesis\BEReBASL\thesis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A93948F-F040-4231-8E4A-4F2EE4B1FB38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F721819-71F3-4893-B411-7FE9E5CA7FDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D47D74D5-B8DF-4140-AD42-DCD0A14E194D}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="126">
   <si>
     <t>Reference</t>
   </si>
@@ -225,9 +225,6 @@
   </si>
   <si>
     <t>MNAR, Bivariate Probit assumptions, FI are rational and may seek to optimize for high balances</t>
-  </si>
-  <si>
-    <t>Emp. and simulation</t>
   </si>
   <si>
     <t>Unclear, only comparision of decision differences presented</t>
@@ -373,6 +370,54 @@
   </si>
   <si>
     <t>Unclear dependency on heuristic distance measures, unclear whether results come from the inferred labels, explainability</t>
+  </si>
+  <si>
+    <t>Xia2019ANR</t>
+  </si>
+  <si>
+    <t>Kang2022CWGAN</t>
+  </si>
+  <si>
+    <t>ribeiro2025balancingperformancerejectinclusion</t>
+  </si>
+  <si>
+    <t>Moderately based on accepts only eval</t>
+  </si>
+  <si>
+    <t>Estimate Isolation Forest (IFO) on rejects to label them: outliers as goods, inliers as bad where this classification happens through heuristic setting of Contamination Rate (CR). Then LightGBM on rejects and accepts where missing values of rejects' features are set to 0 and all features are 0-1 normalized</t>
+  </si>
+  <si>
+    <t>Accurately estimating the true latent contamination rate (CR) of the rejects, as the optimal CR varies between datasets and heavily impacts model performanc</t>
+  </si>
+  <si>
+    <t>MNAR, acceptance decision process is very good: almost only bads are rejected, as IFO-uncommon rejects are expected to be good payers; bads among the rejects are homogenous. 0 imputation is good regardless the type of feature</t>
+  </si>
+  <si>
+    <t>Conditional Wasserstein Generative Adversarial Network with Gradient Penalty (CWGAN-GP) combined with Multi-Task Learning (MTL). First, CWGAN-GP models the complete population feature space using rejects with ``virtual labels''\footnote{The derivation or assignment mechanism for these virtual labels is not explicitly specified in the paper.} to generate synthetic defaults. Second, a multi-task network with shared embedding layers jointly optimizes default risk on the CWGAN-GP-rebalanced dataset and acceptance classification using the rejected features.</t>
+  </si>
+  <si>
+    <t>Likely MNAR\footnote{As they model explicitly the Accept/Reject decision, not explicitly formulated}. Same features among accepts and rejects. Virtual label mechanism for rejects does not bias the generative process and does not need weighting these observations. The same latent feature representations for rejects works for modeling GB and AR equations. That specific AR modeling alleviates the bias on GB.</t>
+  </si>
+  <si>
+    <t>On holdout accept: yes for rebalancing and moderately prediction\footnote{The greatest gain in prediction comes from the rebalancing, the MLT part was not benchmarked to other methods considering auxiliary tasks like Heckman's model}</t>
+  </si>
+  <si>
+    <t>Computational burden of training generative model, selecting the rate of generated samples, explainability</t>
+  </si>
+  <si>
+    <t>Confident Inlier Extrapolation (CI-EX): A semi-supervised framework that iteratively identifies non-outlier rejected samples per class using class-conditional Isolation Forest and assigns labels to the most confident candidates based on probabilities from a balanced classifier</t>
+  </si>
+  <si>
+    <t>Rejects are geomatric inliers relative to accepted samples and can be safely pseudo-labeled using classifier certainty. Iterative, controlled addition of confident inliers prevents catastrophic extrapolation drift. valuating RI solely on accepted test sets (via standard AUC) is fundamentally biased, requiring population/debiased metrics like Kickout and Area Under the Kickout (AUK)</t>
+  </si>
+  <si>
+    <t>Emp. and sim.</t>
+  </si>
+  <si>
+    <t>Moderately / Trade-off dependent</t>
+  </si>
+  <si>
+    <t>Managing the explicit trade-off between maximizing population debiasing (AUK) and maintaining accepted-set accuracy (AUC), alongside the computational overhead of multi-step iterative retraining</t>
   </si>
 </sst>
 </file>
@@ -419,10 +464,8 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -759,695 +802,793 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8852FF5C-5175-44DA-A620-18833DBB2C7A}">
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="38.33203125" customWidth="1"/>
-    <col min="2" max="3" width="28.21875" customWidth="1"/>
-    <col min="4" max="4" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.6640625" customWidth="1"/>
-    <col min="6" max="6" width="28.6640625" customWidth="1"/>
-    <col min="7" max="7" width="24.88671875" customWidth="1"/>
-    <col min="8" max="8" width="27.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.44140625" customWidth="1"/>
-    <col min="10" max="10" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.33203125" style="2" customWidth="1"/>
+    <col min="2" max="3" width="28.21875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="21.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.6640625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="28.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="24.88671875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="27.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.44140625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="27.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="11.5546875" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" t="b">
-        <v>0</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="C2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="1" t="b">
+      <c r="J2" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D3" t="b">
-        <v>1</v>
-      </c>
-      <c r="E3" t="b">
-        <v>0</v>
-      </c>
-      <c r="F3" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="D3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="1" t="b">
+      <c r="J3" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D4" t="b">
-        <v>0</v>
-      </c>
-      <c r="E4" t="b">
-        <v>0</v>
-      </c>
-      <c r="F4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="D4" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="3" t="s">
         <v>14</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="J4" t="b">
+        <v>72</v>
+      </c>
+      <c r="J4" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D5" t="b">
-        <v>1</v>
-      </c>
-      <c r="E5" t="b">
-        <v>1</v>
-      </c>
-      <c r="F5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" t="s">
+      <c r="D5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="J5" t="b">
+      <c r="J5" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D6" t="b">
-        <v>1</v>
-      </c>
-      <c r="E6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="D6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J6" t="b">
+      <c r="J6" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D7" t="b">
-        <v>1</v>
-      </c>
-      <c r="E7" t="b">
-        <v>1</v>
-      </c>
-      <c r="F7" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="D7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J7" t="b">
+      <c r="J7" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="2" t="str">
+      <c r="C8" s="3" t="str">
         <f>"For BVP like in \textcite{"&amp;A7&amp;"}. For Augmentation like \textcite{"&amp;A6&amp;"}"</f>
         <v>For BVP like in \textcite{BanasikCrook2003SampleSelBias}. For Augmentation like \textcite{Banasik01032010}</v>
       </c>
-      <c r="D8" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="E8" t="b">
-        <v>1</v>
-      </c>
-      <c r="F8" t="b">
-        <v>0</v>
-      </c>
-      <c r="G8" t="s">
+      <c r="D8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="2" t="str">
+      <c r="I8" s="3" t="str">
         <f>"Also alike to \textcite{"&amp;A7&amp;"} and \textcite{"&amp;A6&amp;"}"</f>
         <v>Also alike to \textcite{BanasikCrook2003SampleSelBias} and \textcite{Banasik01032010}</v>
       </c>
-      <c r="J8" t="b">
+      <c r="J8" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="2" t="str">
+      <c r="C9" s="3" t="str">
         <f>"For Augmentation like \textcite{"&amp;A6&amp;"}, for extrapolation $\mathbb{P}(Y=g | X)$ similar in accepts and rejects"</f>
         <v>For Augmentation like \textcite{Banasik01032010}, for extrapolation $\mathbb{P}(Y=g | X)$ similar in accepts and rejects</v>
       </c>
-      <c r="D9" t="b">
-        <v>1</v>
-      </c>
-      <c r="E9" t="b">
-        <v>1</v>
-      </c>
-      <c r="F9" t="b">
-        <v>0</v>
-      </c>
-      <c r="G9" t="s">
+      <c r="D9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I9" s="1" t="str">
+      <c r="I9" s="2" t="str">
         <f>"Like \textcite{"&amp;A7&amp;"} and \textcite{"&amp;A6&amp;"}"</f>
         <v>Like \textcite{BanasikCrook2003SampleSelBias} and \textcite{Banasik01032010}</v>
       </c>
-      <c r="J9" t="b">
+      <c r="J9" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="E10" t="b">
-        <v>0</v>
-      </c>
-      <c r="F10" t="b">
-        <v>0</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="D10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F10" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="J10" t="b">
+      <c r="J10" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="A11" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>50</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="D11" t="b">
-        <v>1</v>
-      </c>
-      <c r="E11" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="F11" t="b">
-        <v>0</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="D11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="J11" t="b">
+      <c r="J11" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="72" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>57</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D12" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="E12" t="b">
-        <v>1</v>
-      </c>
-      <c r="F12" t="b">
-        <v>0</v>
-      </c>
-      <c r="G12" t="s">
+      <c r="D12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="I12" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="J12" t="b">
+      <c r="J12" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="72" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="A13" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="J13" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F14" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="J14" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="J15" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="J16" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F17" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="I17" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="J17" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="72" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F18" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="J18" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D19" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F19" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="I19" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="J19" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="D20" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F20" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="I20" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="J20" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="345.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C13" t="s">
-        <v>61</v>
-      </c>
-      <c r="D13" t="b">
-        <v>1</v>
-      </c>
-      <c r="E13" t="b">
-        <v>1</v>
-      </c>
-      <c r="F13" t="b">
-        <v>0</v>
-      </c>
-      <c r="G13" t="s">
-        <v>62</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="J13" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>66</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C14" t="s">
-        <v>68</v>
-      </c>
-      <c r="D14" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="E14" t="b">
-        <v>1</v>
-      </c>
-      <c r="F14" t="b">
-        <v>0</v>
-      </c>
-      <c r="G14" t="s">
-        <v>69</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="J14" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="D15" t="b">
-        <v>0</v>
-      </c>
-      <c r="E15" t="b">
-        <v>0</v>
-      </c>
-      <c r="F15" t="b">
-        <v>1</v>
-      </c>
-      <c r="G15" t="s">
+      <c r="B21" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D21" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E21" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G21" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H15" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="J15" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="201.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D16" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="E16" t="b">
-        <v>1</v>
-      </c>
-      <c r="F16" t="b">
-        <v>0</v>
-      </c>
-      <c r="G16" t="s">
-        <v>78</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="J16" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="D17" t="b">
-        <v>1</v>
-      </c>
-      <c r="E17" t="b">
-        <v>1</v>
-      </c>
-      <c r="F17" t="b">
-        <v>0</v>
-      </c>
-      <c r="G17" t="s">
-        <v>85</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="J17" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="72" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>88</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="D18" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="E18" t="b">
-        <v>1</v>
-      </c>
-      <c r="F18" t="b">
-        <v>0</v>
-      </c>
-      <c r="G18" t="s">
-        <v>91</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="J18" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>94</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="D19" t="b">
-        <v>0</v>
-      </c>
-      <c r="E19" t="b">
-        <v>1</v>
-      </c>
-      <c r="F19" t="b">
-        <v>0</v>
-      </c>
-      <c r="G19" t="s">
+      <c r="H21" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="J21" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="144" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D22" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E22" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="F22" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H19" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="J19" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="187.2" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>100</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="D20" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="E20" t="b">
-        <v>1</v>
-      </c>
-      <c r="F20" t="b">
-        <v>0</v>
-      </c>
-      <c r="G20" t="s">
+      <c r="H22" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="J22" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="273.60000000000002" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D23" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="E23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F23" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="J20" s="1" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="345.6" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>106</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D21" t="b">
-        <v>0</v>
-      </c>
-      <c r="E21" t="b">
-        <v>0</v>
-      </c>
-      <c r="F21" t="b">
-        <v>1</v>
-      </c>
-      <c r="G21" t="s">
-        <v>22</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="J21" t="b">
-        <v>0</v>
-      </c>
+      <c r="H23" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="J23" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F24" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="I24" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="J24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="K24" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>